<commit_message>
Trying to add subsidy on wind on shore
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_tariffs_and_subsidies.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_tariffs_and_subsidies.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0501804-ED93-4344-A61C-67BD67E17E87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C02A2D6-4E2C-4C9E-B09A-BF4278813E22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,10 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
-  <si>
-    <t>Pset_Set</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Pset_PN</t>
   </si>
@@ -56,16 +53,16 @@
     <t>LimType</t>
   </si>
   <si>
-    <t>windon,windoff</t>
-  </si>
-  <si>
     <t>~TFM_INS</t>
   </si>
   <si>
-    <t>Other_Indexes</t>
-  </si>
-  <si>
     <t>FLO_SUB</t>
+  </si>
+  <si>
+    <t>Process</t>
+  </si>
+  <si>
+    <t>E[_]WON*</t>
   </si>
 </sst>
 </file>
@@ -173,8 +170,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="3" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="4"/>
@@ -474,7 +470,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:M6"/>
+  <dimension ref="B2:J6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="24.28515625" bestFit="1" customWidth="1"/>
@@ -483,92 +479,67 @@
     <col min="6" max="6" width="18.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B2" s="2"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
+    <row r="2" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B2" s="1"/>
     </row>
-    <row r="3" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B3" s="2"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
-      <c r="M3" s="1"/>
+    <row r="3" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B3" s="1"/>
     </row>
-    <row r="4" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B4" s="3"/>
-      <c r="C4" s="6" t="s">
+    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B4" s="2"/>
+      <c r="C4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+    </row>
+    <row r="5" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" s="7">
+        <v>2025</v>
+      </c>
+      <c r="E5" s="7">
+        <v>2030</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
+      <c r="G5" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="J5" s="6">
+        <v>0</v>
+      </c>
     </row>
-    <row r="5" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="8">
-        <v>2025</v>
-      </c>
-      <c r="F5" s="8">
-        <v>2030</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="J5" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="K5" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
-        <v>9</v>
+        <v>6</v>
+      </c>
+      <c r="D6">
+        <v>8.4</v>
       </c>
       <c r="E6">
         <v>8.4</v>
       </c>
-      <c r="F6">
-        <v>8.4</v>
-      </c>
-      <c r="I6" t="s">
-        <v>6</v>
-      </c>
-      <c r="K6">
+      <c r="F6" t="s">
+        <v>8</v>
+      </c>
+      <c r="J6">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Correction on subsidy declaration
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_tariffs_and_subsidies.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_tariffs_and_subsidies.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AED91FA2-267C-450C-A109-EA81C4D4BA70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2ADCAD8-E106-4FD3-90D1-DD1D5F8E736A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,9 +41,6 @@
     <t>Attribute</t>
   </si>
   <si>
-    <t>~TFM_INS</t>
-  </si>
-  <si>
     <t>FLO_SUB</t>
   </si>
   <si>
@@ -57,6 +54,9 @@
   </si>
   <si>
     <t>ELC</t>
+  </si>
+  <si>
+    <t>~TFM_INS-TS</t>
   </si>
 </sst>
 </file>
@@ -459,7 +459,7 @@
   <dimension ref="B4:I6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.6328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.1796875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.453125" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="4.81640625" bestFit="1" customWidth="1"/>
@@ -467,7 +467,7 @@
   <sheetData>
     <row r="4" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B4" s="4" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
@@ -482,10 +482,10 @@
         <v>0</v>
       </c>
       <c r="C5" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>4</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>5</v>
       </c>
       <c r="E5" s="3">
         <v>2025</v>
@@ -499,13 +499,13 @@
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
         <v>2</v>
       </c>
-      <c r="C6" t="s">
-        <v>3</v>
-      </c>
       <c r="D6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E6">
         <v>8.4</v>

</xml_diff>